<commit_message>
Continuing to clean up the main figures
</commit_message>
<xml_diff>
--- a/data/compendium_library_depth.xlsx
+++ b/data/compendium_library_depth.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/annaleigh/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/annaleigh/Documents/GitHub/online/cryptic_biology/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B153551-5647-584C-B0BD-1F4715647179}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DAA0C4B5-E94B-B348-AC82-BE29F319092F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17520" activeTab="1" xr2:uid="{F3336A91-2557-674F-B064-F692FFC423CD}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17520" xr2:uid="{F3336A91-2557-674F-B064-F692FFC423CD}"/>
   </bookViews>
   <sheets>
     <sheet name="Compendium" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="216" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="255" uniqueCount="110">
   <si>
     <t>sample</t>
   </si>
@@ -323,6 +323,51 @@
   </si>
   <si>
     <t>SK-N-BE(2) curve</t>
+  </si>
+  <si>
+    <t>Cont-A_S1.pass2Aligned.sortedByCoord.out.bam</t>
+  </si>
+  <si>
+    <t>Cont-B_S2.pass2Aligned.sortedByCoord.out.bam</t>
+  </si>
+  <si>
+    <t>Cont-C_S3.pass2Aligned.sortedByCoord.out.bam</t>
+  </si>
+  <si>
+    <t>Cont-D_S4.pass2Aligned.sortedByCoord.out.bam</t>
+  </si>
+  <si>
+    <t>TDP43-E_S5.pass2Aligned.sortedByCoord.out.bam</t>
+  </si>
+  <si>
+    <t>TDP43-F_S6.pass2Aligned.sortedByCoord.out.bam</t>
+  </si>
+  <si>
+    <t>TDP43-G_S7.pass2Aligned.sortedByCoord.out.bam</t>
+  </si>
+  <si>
+    <t>Brown-SHSY5Y</t>
+  </si>
+  <si>
+    <t>CTR07.Aligned.sorted.out.bam</t>
+  </si>
+  <si>
+    <t>CTR08.Aligned.sorted.out.bam</t>
+  </si>
+  <si>
+    <t>CTR09.Aligned.sorted.out.bam</t>
+  </si>
+  <si>
+    <t>TDP10.Aligned.sorted.out.bam</t>
+  </si>
+  <si>
+    <t>TDP11.Aligned.sorted.out.bam</t>
+  </si>
+  <si>
+    <t>TDP12.Aligned.sorted.out.bam</t>
+  </si>
+  <si>
+    <t>Brown-SKNBE2</t>
   </si>
 </sst>
 </file>
@@ -376,10 +421,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -717,7 +761,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7FAB4AF4-1493-4F4C-9D24-CCB1BDE91B2C}">
-  <dimension ref="A1:D30"/>
+  <dimension ref="A1:D43"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="63.1640625" bestFit="1" customWidth="1"/>
@@ -726,10 +770,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A1" s="2" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
       <c r="C1" t="s">
@@ -740,10 +784,10 @@
       </c>
     </row>
     <row r="2" spans="1:4" ht="22" x14ac:dyDescent="0.25">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="2">
+      <c r="B2">
         <v>52326116</v>
       </c>
       <c r="C2" t="s">
@@ -754,10 +798,10 @@
       </c>
     </row>
     <row r="3" spans="1:4" ht="22" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="2">
+      <c r="B3">
         <v>48866512</v>
       </c>
       <c r="C3" t="s">
@@ -768,10 +812,10 @@
       </c>
     </row>
     <row r="4" spans="1:4" ht="22" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="2">
+      <c r="B4">
         <v>54180349</v>
       </c>
       <c r="C4" t="s">
@@ -782,10 +826,10 @@
       </c>
     </row>
     <row r="5" spans="1:4" ht="22" x14ac:dyDescent="0.25">
-      <c r="A5" s="3" t="s">
+      <c r="A5" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="2">
+      <c r="B5">
         <v>45151956</v>
       </c>
       <c r="C5" t="s">
@@ -796,10 +840,10 @@
       </c>
     </row>
     <row r="6" spans="1:4" ht="22" x14ac:dyDescent="0.25">
-      <c r="A6" s="3" t="s">
+      <c r="A6" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B6" s="2">
+      <c r="B6">
         <v>50783887</v>
       </c>
       <c r="C6" t="s">
@@ -810,10 +854,10 @@
       </c>
     </row>
     <row r="7" spans="1:4" ht="22" x14ac:dyDescent="0.25">
-      <c r="A7" s="3" t="s">
+      <c r="A7" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B7" s="2">
+      <c r="B7">
         <v>46430080</v>
       </c>
       <c r="C7" t="s">
@@ -824,10 +868,10 @@
       </c>
     </row>
     <row r="8" spans="1:4" ht="22" x14ac:dyDescent="0.25">
-      <c r="A8" s="3" t="s">
+      <c r="A8" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B8" s="2">
+      <c r="B8">
         <v>45683362</v>
       </c>
       <c r="C8" t="s">
@@ -838,10 +882,10 @@
       </c>
     </row>
     <row r="9" spans="1:4" ht="22" x14ac:dyDescent="0.25">
-      <c r="A9" s="3" t="s">
+      <c r="A9" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B9" s="2">
+      <c r="B9">
         <v>49002563</v>
       </c>
       <c r="C9" t="s">
@@ -852,10 +896,10 @@
       </c>
     </row>
     <row r="10" spans="1:4" ht="22" x14ac:dyDescent="0.25">
-      <c r="A10" s="3" t="s">
+      <c r="A10" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B10" s="2">
+      <c r="B10">
         <v>49330182</v>
       </c>
       <c r="C10" t="s">
@@ -866,10 +910,10 @@
       </c>
     </row>
     <row r="11" spans="1:4" ht="22" x14ac:dyDescent="0.25">
-      <c r="A11" s="3" t="s">
+      <c r="A11" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B11" s="2">
+      <c r="B11">
         <v>56653582</v>
       </c>
       <c r="C11" t="s">
@@ -880,10 +924,10 @@
       </c>
     </row>
     <row r="12" spans="1:4" ht="22" x14ac:dyDescent="0.25">
-      <c r="A12" s="3" t="s">
+      <c r="A12" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B12" s="2">
+      <c r="B12">
         <v>43366558</v>
       </c>
       <c r="C12" t="s">
@@ -894,10 +938,10 @@
       </c>
     </row>
     <row r="13" spans="1:4" ht="22" x14ac:dyDescent="0.25">
-      <c r="A13" s="3" t="s">
+      <c r="A13" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B13" s="2">
+      <c r="B13">
         <v>46685686</v>
       </c>
       <c r="C13" t="s">
@@ -908,10 +952,10 @@
       </c>
     </row>
     <row r="14" spans="1:4" ht="22" x14ac:dyDescent="0.25">
-      <c r="A14" s="3" t="s">
+      <c r="A14" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B14" s="2">
+      <c r="B14">
         <v>49805939</v>
       </c>
       <c r="C14" t="s">
@@ -922,10 +966,10 @@
       </c>
     </row>
     <row r="15" spans="1:4" ht="22" x14ac:dyDescent="0.25">
-      <c r="A15" s="3" t="s">
+      <c r="A15" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B15" s="2">
+      <c r="B15">
         <v>52803386</v>
       </c>
       <c r="C15" t="s">
@@ -936,10 +980,10 @@
       </c>
     </row>
     <row r="16" spans="1:4" ht="22" x14ac:dyDescent="0.25">
-      <c r="A16" s="3" t="s">
+      <c r="A16" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="B16" s="2">
+      <c r="B16">
         <v>47016967</v>
       </c>
       <c r="C16" t="s">
@@ -950,10 +994,10 @@
       </c>
     </row>
     <row r="17" spans="1:4" ht="22" x14ac:dyDescent="0.25">
-      <c r="A17" s="3" t="s">
+      <c r="A17" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B17" s="2">
+      <c r="B17">
         <v>45596326</v>
       </c>
       <c r="C17" t="s">
@@ -1057,7 +1101,7 @@
       <c r="C24" t="s">
         <v>19</v>
       </c>
-      <c r="D24" s="4" t="s">
+      <c r="D24" s="3" t="s">
         <v>30</v>
       </c>
     </row>
@@ -1071,7 +1115,7 @@
       <c r="C25" t="s">
         <v>19</v>
       </c>
-      <c r="D25" s="4" t="s">
+      <c r="D25" s="3" t="s">
         <v>30</v>
       </c>
     </row>
@@ -1085,7 +1129,7 @@
       <c r="C26" t="s">
         <v>19</v>
       </c>
-      <c r="D26" s="4" t="s">
+      <c r="D26" s="3" t="s">
         <v>30</v>
       </c>
     </row>
@@ -1099,7 +1143,7 @@
       <c r="C27" t="s">
         <v>20</v>
       </c>
-      <c r="D27" s="4" t="s">
+      <c r="D27" s="3" t="s">
         <v>30</v>
       </c>
     </row>
@@ -1113,7 +1157,7 @@
       <c r="C28" t="s">
         <v>20</v>
       </c>
-      <c r="D28" s="4" t="s">
+      <c r="D28" s="3" t="s">
         <v>30</v>
       </c>
     </row>
@@ -1127,13 +1171,195 @@
       <c r="C29" t="s">
         <v>20</v>
       </c>
-      <c r="D29" s="4" t="s">
+      <c r="D29" s="3" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:4" ht="22" x14ac:dyDescent="0.25">
+      <c r="A30" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="B30">
+        <v>47514679</v>
+      </c>
+      <c r="C30" t="s">
+        <v>19</v>
+      </c>
       <c r="D30" t="s">
         <v>37</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" ht="22" x14ac:dyDescent="0.25">
+      <c r="A31" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="B31">
+        <v>69168102</v>
+      </c>
+      <c r="C31" t="s">
+        <v>19</v>
+      </c>
+      <c r="D31" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" ht="22" x14ac:dyDescent="0.25">
+      <c r="A32" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="B32">
+        <v>43555020</v>
+      </c>
+      <c r="C32" t="s">
+        <v>19</v>
+      </c>
+      <c r="D32" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" ht="22" x14ac:dyDescent="0.25">
+      <c r="A33" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="B33">
+        <v>54609711</v>
+      </c>
+      <c r="C33" t="s">
+        <v>19</v>
+      </c>
+      <c r="D33" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" ht="22" x14ac:dyDescent="0.25">
+      <c r="A34" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="B34">
+        <v>47687085</v>
+      </c>
+      <c r="C34" t="s">
+        <v>20</v>
+      </c>
+      <c r="D34" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" ht="22" x14ac:dyDescent="0.25">
+      <c r="A35" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="B35">
+        <v>53658704</v>
+      </c>
+      <c r="C35" t="s">
+        <v>20</v>
+      </c>
+      <c r="D35" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" ht="22" x14ac:dyDescent="0.25">
+      <c r="A36" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="B36">
+        <v>49860423</v>
+      </c>
+      <c r="C36" t="s">
+        <v>20</v>
+      </c>
+      <c r="D36" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" ht="22" x14ac:dyDescent="0.25">
+      <c r="A37" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="B37">
+        <v>68914513</v>
+      </c>
+      <c r="C37" t="s">
+        <v>19</v>
+      </c>
+      <c r="D37" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" ht="22" x14ac:dyDescent="0.25">
+      <c r="A38" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="B38">
+        <v>61890171</v>
+      </c>
+      <c r="C38" t="s">
+        <v>19</v>
+      </c>
+      <c r="D38" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" ht="22" x14ac:dyDescent="0.25">
+      <c r="A39" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="B39">
+        <v>56711754</v>
+      </c>
+      <c r="C39" t="s">
+        <v>19</v>
+      </c>
+      <c r="D39" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" ht="22" x14ac:dyDescent="0.25">
+      <c r="A40" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="B40">
+        <v>60098925</v>
+      </c>
+      <c r="C40" t="s">
+        <v>20</v>
+      </c>
+      <c r="D40" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" ht="22" x14ac:dyDescent="0.25">
+      <c r="A41" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="B41">
+        <v>58436114</v>
+      </c>
+      <c r="C41" t="s">
+        <v>20</v>
+      </c>
+      <c r="D41" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" ht="22" x14ac:dyDescent="0.25">
+      <c r="A42" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="B42">
+        <v>63384713</v>
+      </c>
+      <c r="C42" t="s">
+        <v>20</v>
+      </c>
+      <c r="D42" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="D43" t="s">
+        <v>109</v>
       </c>
     </row>
   </sheetData>
@@ -1148,17 +1374,17 @@
   <cols>
     <col min="1" max="1" width="73.5" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="15.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.83203125" style="5"/>
+    <col min="3" max="3" width="10.83203125" style="4"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A1" s="2" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="C1" s="4" t="s">
         <v>62</v>
       </c>
       <c r="D1" t="s">
@@ -1172,7 +1398,7 @@
       <c r="B2">
         <v>45612319</v>
       </c>
-      <c r="C2" s="5" t="s">
+      <c r="C2" s="4" t="s">
         <v>58</v>
       </c>
       <c r="D2" t="s">
@@ -1186,7 +1412,7 @@
       <c r="B3">
         <v>45036466</v>
       </c>
-      <c r="C3" s="5" t="s">
+      <c r="C3" s="4" t="s">
         <v>58</v>
       </c>
       <c r="D3" t="s">
@@ -1200,7 +1426,7 @@
       <c r="B4">
         <v>47094977</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="C4" s="4" t="s">
         <v>58</v>
       </c>
       <c r="D4" t="s">
@@ -1214,7 +1440,7 @@
       <c r="B5">
         <v>42133698</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="C5" s="4" t="s">
         <v>59</v>
       </c>
       <c r="D5" t="s">
@@ -1228,7 +1454,7 @@
       <c r="B6">
         <v>42635436</v>
       </c>
-      <c r="C6" s="5" t="s">
+      <c r="C6" s="4" t="s">
         <v>59</v>
       </c>
       <c r="D6" t="s">
@@ -1242,7 +1468,7 @@
       <c r="B7">
         <v>44092088</v>
       </c>
-      <c r="C7" s="5" t="s">
+      <c r="C7" s="4" t="s">
         <v>59</v>
       </c>
       <c r="D7" t="s">
@@ -1256,7 +1482,7 @@
       <c r="B8">
         <v>43803894</v>
       </c>
-      <c r="C8" s="5" t="s">
+      <c r="C8" s="4" t="s">
         <v>60</v>
       </c>
       <c r="D8" t="s">
@@ -1270,7 +1496,7 @@
       <c r="B9">
         <v>42635436</v>
       </c>
-      <c r="C9" s="5" t="s">
+      <c r="C9" s="4" t="s">
         <v>60</v>
       </c>
       <c r="D9" t="s">
@@ -1284,7 +1510,7 @@
       <c r="B10">
         <v>41746651</v>
       </c>
-      <c r="C10" s="5" t="s">
+      <c r="C10" s="4" t="s">
         <v>60</v>
       </c>
       <c r="D10" t="s">
@@ -1298,7 +1524,7 @@
       <c r="B11">
         <v>43612293</v>
       </c>
-      <c r="C11" s="5" t="s">
+      <c r="C11" s="4" t="s">
         <v>61</v>
       </c>
       <c r="D11" t="s">
@@ -1312,7 +1538,7 @@
       <c r="B12">
         <v>48002107</v>
       </c>
-      <c r="C12" s="5" t="s">
+      <c r="C12" s="4" t="s">
         <v>61</v>
       </c>
       <c r="D12" t="s">
@@ -1326,7 +1552,7 @@
       <c r="B13">
         <v>44693558</v>
       </c>
-      <c r="C13" s="5" t="s">
+      <c r="C13" s="4" t="s">
         <v>61</v>
       </c>
       <c r="D13" t="s">
@@ -1340,7 +1566,7 @@
       <c r="B14">
         <v>45380071</v>
       </c>
-      <c r="C14" s="5" t="s">
+      <c r="C14" s="4" t="s">
         <v>57</v>
       </c>
       <c r="D14" t="s">
@@ -1354,7 +1580,7 @@
       <c r="B15">
         <v>35295930</v>
       </c>
-      <c r="C15" s="5" t="s">
+      <c r="C15" s="4" t="s">
         <v>57</v>
       </c>
       <c r="D15" t="s">
@@ -1368,7 +1594,7 @@
       <c r="B16">
         <v>35255210</v>
       </c>
-      <c r="C16" s="5" t="s">
+      <c r="C16" s="4" t="s">
         <v>57</v>
       </c>
       <c r="D16" t="s">
@@ -1382,7 +1608,7 @@
       <c r="B17">
         <v>42817897</v>
       </c>
-      <c r="C17" s="5">
+      <c r="C17" s="4">
         <v>0</v>
       </c>
       <c r="D17" t="s">
@@ -1396,7 +1622,7 @@
       <c r="B18">
         <v>42639282</v>
       </c>
-      <c r="C18" s="5">
+      <c r="C18" s="4">
         <v>0</v>
       </c>
       <c r="D18" t="s">
@@ -1410,7 +1636,7 @@
       <c r="B19">
         <v>46653407</v>
       </c>
-      <c r="C19" s="5">
+      <c r="C19" s="4">
         <v>0</v>
       </c>
       <c r="D19" t="s">
@@ -1424,7 +1650,7 @@
       <c r="B20">
         <v>59722789</v>
       </c>
-      <c r="C20" s="5" t="s">
+      <c r="C20" s="4" t="s">
         <v>89</v>
       </c>
       <c r="D20" t="s">
@@ -1438,7 +1664,7 @@
       <c r="B21">
         <v>60580872</v>
       </c>
-      <c r="C21" s="5" t="s">
+      <c r="C21" s="4" t="s">
         <v>89</v>
       </c>
       <c r="D21" t="s">
@@ -1452,7 +1678,7 @@
       <c r="B22">
         <v>64852515</v>
       </c>
-      <c r="C22" s="5" t="s">
+      <c r="C22" s="4" t="s">
         <v>89</v>
       </c>
       <c r="D22" t="s">
@@ -1466,7 +1692,7 @@
       <c r="B23">
         <v>57407638</v>
       </c>
-      <c r="C23" s="5" t="s">
+      <c r="C23" s="4" t="s">
         <v>90</v>
       </c>
       <c r="D23" t="s">
@@ -1480,7 +1706,7 @@
       <c r="B24">
         <v>55116047</v>
       </c>
-      <c r="C24" s="5" t="s">
+      <c r="C24" s="4" t="s">
         <v>90</v>
       </c>
       <c r="D24" t="s">
@@ -1494,7 +1720,7 @@
       <c r="B25">
         <v>60662949</v>
       </c>
-      <c r="C25" s="5" t="s">
+      <c r="C25" s="4" t="s">
         <v>90</v>
       </c>
       <c r="D25" t="s">
@@ -1508,7 +1734,7 @@
       <c r="B26">
         <v>62421518</v>
       </c>
-      <c r="C26" s="5" t="s">
+      <c r="C26" s="4" t="s">
         <v>91</v>
       </c>
       <c r="D26" t="s">
@@ -1522,7 +1748,7 @@
       <c r="B27">
         <v>60057543</v>
       </c>
-      <c r="C27" s="5" t="s">
+      <c r="C27" s="4" t="s">
         <v>91</v>
       </c>
       <c r="D27" t="s">
@@ -1536,7 +1762,7 @@
       <c r="B28">
         <v>68751836</v>
       </c>
-      <c r="C28" s="5" t="s">
+      <c r="C28" s="4" t="s">
         <v>91</v>
       </c>
       <c r="D28" t="s">
@@ -1550,7 +1776,7 @@
       <c r="B29">
         <v>62555837</v>
       </c>
-      <c r="C29" s="5" t="s">
+      <c r="C29" s="4" t="s">
         <v>92</v>
       </c>
       <c r="D29" t="s">
@@ -1564,7 +1790,7 @@
       <c r="B30">
         <v>53910345</v>
       </c>
-      <c r="C30" s="5" t="s">
+      <c r="C30" s="4" t="s">
         <v>92</v>
       </c>
       <c r="D30" t="s">
@@ -1578,7 +1804,7 @@
       <c r="B31">
         <v>61823241</v>
       </c>
-      <c r="C31" s="5" t="s">
+      <c r="C31" s="4" t="s">
         <v>92</v>
       </c>
       <c r="D31" t="s">
@@ -1592,7 +1818,7 @@
       <c r="B32">
         <v>55259391</v>
       </c>
-      <c r="C32" s="5" t="s">
+      <c r="C32" s="4" t="s">
         <v>57</v>
       </c>
       <c r="D32" t="s">
@@ -1606,7 +1832,7 @@
       <c r="B33">
         <v>68567792</v>
       </c>
-      <c r="C33" s="5" t="s">
+      <c r="C33" s="4" t="s">
         <v>57</v>
       </c>
       <c r="D33" t="s">
@@ -1620,7 +1846,7 @@
       <c r="B34">
         <v>76895715</v>
       </c>
-      <c r="C34" s="5" t="s">
+      <c r="C34" s="4" t="s">
         <v>57</v>
       </c>
       <c r="D34" t="s">
@@ -1634,7 +1860,7 @@
       <c r="B35">
         <v>71271129</v>
       </c>
-      <c r="C35" s="5" t="s">
+      <c r="C35" s="4" t="s">
         <v>93</v>
       </c>
       <c r="D35" t="s">
@@ -1648,7 +1874,7 @@
       <c r="B36">
         <v>63051148</v>
       </c>
-      <c r="C36" s="5" t="s">
+      <c r="C36" s="4" t="s">
         <v>93</v>
       </c>
       <c r="D36" t="s">
@@ -1662,7 +1888,7 @@
       <c r="B37">
         <v>59380615</v>
       </c>
-      <c r="C37" s="5" t="s">
+      <c r="C37" s="4" t="s">
         <v>93</v>
       </c>
       <c r="D37" t="s">
@@ -1676,7 +1902,7 @@
       <c r="B38">
         <v>57679461</v>
       </c>
-      <c r="C38" s="5" t="s">
+      <c r="C38" s="4" t="s">
         <v>88</v>
       </c>
       <c r="D38" t="s">
@@ -1690,7 +1916,7 @@
       <c r="B39">
         <v>60402144</v>
       </c>
-      <c r="C39" s="5" t="s">
+      <c r="C39" s="4" t="s">
         <v>88</v>
       </c>
       <c r="D39" t="s">
@@ -1704,7 +1930,7 @@
       <c r="B40">
         <v>56967532</v>
       </c>
-      <c r="C40" s="5" t="s">
+      <c r="C40" s="4" t="s">
         <v>88</v>
       </c>
       <c r="D40" t="s">
@@ -1718,7 +1944,7 @@
       <c r="B41">
         <v>67683062</v>
       </c>
-      <c r="C41" s="5" t="s">
+      <c r="C41" s="4" t="s">
         <v>87</v>
       </c>
       <c r="D41" t="s">
@@ -1732,7 +1958,7 @@
       <c r="B42">
         <v>64707816</v>
       </c>
-      <c r="C42" s="5" t="s">
+      <c r="C42" s="4" t="s">
         <v>87</v>
       </c>
       <c r="D42" t="s">
@@ -1746,7 +1972,7 @@
       <c r="B43">
         <v>64112046</v>
       </c>
-      <c r="C43" s="5" t="s">
+      <c r="C43" s="4" t="s">
         <v>87</v>
       </c>
       <c r="D43" t="s">

</xml_diff>